<commit_message>
Update CW data 2026-08-25
</commit_message>
<xml_diff>
--- a/docs/downloads/ThongTinChungQuyen_latest.xlsx
+++ b/docs/downloads/ThongTinChungQuyen_latest.xlsx
@@ -813,7 +813,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>CTCP Chứng khoán LPBank ( LPS )</t>
+          <t>CTCP Chứng khoán LPS ( LPS )</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>CTCP Chứng khoán LPBank ( LPS )</t>
+          <t>CTCP Chứng khoán LPS ( LPS )</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -3585,7 +3585,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>CTCP Chứng khoán LPBank ( LPS )</t>
+          <t>CTCP Chứng khoán LPS ( LPS )</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -5349,7 +5349,7 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>CTCP Chứng khoán LPBank ( LPS )</t>
+          <t>CTCP Chứng khoán LPS ( LPS )</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
@@ -6021,7 +6021,7 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>CTCP Chứng khoán LPBank ( LPS )</t>
+          <t>CTCP Chứng khoán LPS ( LPS )</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
@@ -11019,7 +11019,7 @@
       </c>
       <c r="B252" s="2" t="inlineStr">
         <is>
-          <t>CTCP Chứng khoán LPBank ( LPS )</t>
+          <t>CTCP Chứng khoán LPS ( LPS )</t>
         </is>
       </c>
       <c r="C252" s="2" t="inlineStr">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B264" s="2" t="inlineStr">
         <is>
-          <t>CTCP Chứng khoán LPBank ( LPS )</t>
+          <t>CTCP Chứng khoán LPS ( LPS )</t>
         </is>
       </c>
       <c r="C264" s="2" t="inlineStr">
@@ -12489,7 +12489,7 @@
       </c>
       <c r="B287" s="2" t="inlineStr">
         <is>
-          <t>CTCP Chứng khoán LPBank ( LPS )</t>
+          <t>CTCP Chứng khoán LPS ( LPS )</t>
         </is>
       </c>
       <c r="C287" s="2" t="inlineStr">

</xml_diff>